<commit_message>
Add earth dam BC2 seepage inputs and update levee files
Add new earth dam BC2 input files with mesh and seepage solutions.
Update levee1 seepage data and levee2 Excel file. Remove obsolete
levee1 mesh JSON (replaced by levee2 mesh). Add levee2 mesh and
seepage CSV.

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/seep/files/xslope_levee2.xlsx
+++ b/docs/seep/files/xslope_levee2.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10102"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10215"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/njones/python_projects/xslope/docs/seep/files/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{82D440DC-91EF-1E4E-8ABD-64EB1023CF02}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{87100ED1-BD7E-914C-99F0-63C98405611C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="27220" yWindow="2900" windowWidth="34200" windowHeight="20240" xr2:uid="{BA54C293-CE08-6E4C-9212-B3317DAA148E}"/>
+    <workbookView xWindow="28520" yWindow="4820" windowWidth="34200" windowHeight="20240" activeTab="2" xr2:uid="{BA54C293-CE08-6E4C-9212-B3317DAA148E}"/>
   </bookViews>
   <sheets>
     <sheet name="main" sheetId="1" r:id="rId1"/>
@@ -1053,13 +1053,13 @@
     <xf numFmtId="0" fontId="10" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="15" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="15" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
@@ -10303,74 +10303,74 @@
       </c>
     </row>
     <row r="4" spans="1:44" x14ac:dyDescent="0.2">
-      <c r="A4" s="45" t="s">
+      <c r="A4" s="47" t="s">
         <v>2</v>
       </c>
-      <c r="B4" s="45"/>
-      <c r="D4" s="45" t="s">
+      <c r="B4" s="47"/>
+      <c r="D4" s="47" t="s">
         <v>5</v>
       </c>
-      <c r="E4" s="45"/>
-      <c r="G4" s="45" t="s">
+      <c r="E4" s="47"/>
+      <c r="G4" s="47" t="s">
         <v>6</v>
       </c>
-      <c r="H4" s="45"/>
-      <c r="J4" s="45" t="s">
+      <c r="H4" s="47"/>
+      <c r="J4" s="47" t="s">
         <v>7</v>
       </c>
-      <c r="K4" s="45"/>
-      <c r="M4" s="45" t="s">
+      <c r="K4" s="47"/>
+      <c r="M4" s="47" t="s">
         <v>8</v>
       </c>
-      <c r="N4" s="45"/>
-      <c r="P4" s="45" t="s">
+      <c r="N4" s="47"/>
+      <c r="P4" s="47" t="s">
         <v>9</v>
       </c>
-      <c r="Q4" s="45"/>
+      <c r="Q4" s="47"/>
       <c r="R4" s="1"/>
-      <c r="S4" s="45" t="s">
+      <c r="S4" s="47" t="s">
         <v>10</v>
       </c>
-      <c r="T4" s="45"/>
+      <c r="T4" s="47"/>
       <c r="U4" s="1"/>
-      <c r="V4" s="45" t="s">
+      <c r="V4" s="47" t="s">
         <v>11</v>
       </c>
-      <c r="W4" s="45"/>
+      <c r="W4" s="47"/>
       <c r="X4" s="1"/>
-      <c r="Y4" s="45" t="s">
+      <c r="Y4" s="47" t="s">
         <v>12</v>
       </c>
-      <c r="Z4" s="45"/>
+      <c r="Z4" s="47"/>
       <c r="AA4" s="1"/>
-      <c r="AB4" s="45" t="s">
+      <c r="AB4" s="47" t="s">
         <v>13</v>
       </c>
-      <c r="AC4" s="45"/>
-      <c r="AE4" s="45" t="s">
+      <c r="AC4" s="47"/>
+      <c r="AE4" s="47" t="s">
         <v>116</v>
       </c>
-      <c r="AF4" s="45"/>
+      <c r="AF4" s="47"/>
       <c r="AG4" s="1"/>
-      <c r="AH4" s="45" t="s">
+      <c r="AH4" s="47" t="s">
         <v>117</v>
       </c>
-      <c r="AI4" s="45"/>
+      <c r="AI4" s="47"/>
       <c r="AJ4" s="1"/>
-      <c r="AK4" s="45" t="s">
+      <c r="AK4" s="47" t="s">
         <v>118</v>
       </c>
-      <c r="AL4" s="45"/>
+      <c r="AL4" s="47"/>
       <c r="AM4" s="1"/>
-      <c r="AN4" s="45" t="s">
+      <c r="AN4" s="47" t="s">
         <v>119</v>
       </c>
-      <c r="AO4" s="45"/>
+      <c r="AO4" s="47"/>
       <c r="AP4" s="1"/>
-      <c r="AQ4" s="45" t="s">
+      <c r="AQ4" s="47" t="s">
         <v>120</v>
       </c>
-      <c r="AR4" s="45"/>
+      <c r="AR4" s="47"/>
     </row>
     <row r="5" spans="1:44" x14ac:dyDescent="0.2">
       <c r="A5" s="41" t="s">
@@ -10473,89 +10473,89 @@
       </c>
     </row>
     <row r="6" spans="1:44" x14ac:dyDescent="0.2">
-      <c r="A6" s="46" t="str">
+      <c r="A6" s="45" t="str">
         <f>_xlfn.XLOOKUP(B5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v>foundation</v>
       </c>
-      <c r="B6" s="47"/>
-      <c r="D6" s="46" t="str">
+      <c r="B6" s="46"/>
+      <c r="D6" s="45" t="str">
         <f>_xlfn.XLOOKUP(E5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v>grout</v>
       </c>
-      <c r="E6" s="47"/>
-      <c r="G6" s="46" t="str">
+      <c r="E6" s="46"/>
+      <c r="G6" s="45" t="str">
         <f>_xlfn.XLOOKUP(H5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v>foundation</v>
       </c>
-      <c r="H6" s="47"/>
-      <c r="J6" s="46" t="str">
+      <c r="H6" s="46"/>
+      <c r="J6" s="45" t="str">
         <f>_xlfn.XLOOKUP(K5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="K6" s="47"/>
-      <c r="M6" s="46" t="str">
+      <c r="K6" s="46"/>
+      <c r="M6" s="45" t="str">
         <f>_xlfn.XLOOKUP(N5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="N6" s="47"/>
-      <c r="P6" s="46" t="str">
+      <c r="N6" s="46"/>
+      <c r="P6" s="45" t="str">
         <f>_xlfn.XLOOKUP(Q5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="Q6" s="47"/>
+      <c r="Q6" s="46"/>
       <c r="R6" s="1"/>
-      <c r="S6" s="46" t="str">
+      <c r="S6" s="45" t="str">
         <f>_xlfn.XLOOKUP(T5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="T6" s="47"/>
+      <c r="T6" s="46"/>
       <c r="U6" s="1"/>
-      <c r="V6" s="46" t="str">
+      <c r="V6" s="45" t="str">
         <f>_xlfn.XLOOKUP(W5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="W6" s="47"/>
+      <c r="W6" s="46"/>
       <c r="X6" s="1"/>
-      <c r="Y6" s="46" t="str">
+      <c r="Y6" s="45" t="str">
         <f>_xlfn.XLOOKUP(Z5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="Z6" s="47"/>
+      <c r="Z6" s="46"/>
       <c r="AA6" s="1"/>
-      <c r="AB6" s="46" t="str">
+      <c r="AB6" s="45" t="str">
         <f>_xlfn.XLOOKUP(AC5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="AC6" s="47"/>
-      <c r="AE6" s="46" t="str">
+      <c r="AC6" s="46"/>
+      <c r="AE6" s="45" t="str">
         <f>_xlfn.XLOOKUP(AF5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="AF6" s="47"/>
+      <c r="AF6" s="46"/>
       <c r="AG6" s="1"/>
-      <c r="AH6" s="46" t="str">
+      <c r="AH6" s="45" t="str">
         <f>_xlfn.XLOOKUP(AI5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="AI6" s="47"/>
+      <c r="AI6" s="46"/>
       <c r="AJ6" s="1"/>
-      <c r="AK6" s="46" t="str">
+      <c r="AK6" s="45" t="str">
         <f>_xlfn.XLOOKUP(AL5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="AL6" s="47"/>
+      <c r="AL6" s="46"/>
       <c r="AM6" s="1"/>
-      <c r="AN6" s="46" t="str">
+      <c r="AN6" s="45" t="str">
         <f>_xlfn.XLOOKUP(AO5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="AO6" s="47"/>
+      <c r="AO6" s="46"/>
       <c r="AP6" s="1"/>
-      <c r="AQ6" s="46" t="str">
+      <c r="AQ6" s="45" t="str">
         <f>_xlfn.XLOOKUP(AR5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="AR6" s="47"/>
+      <c r="AR6" s="46"/>
     </row>
     <row r="7" spans="1:44" x14ac:dyDescent="0.2">
       <c r="A7" s="2" t="s">
@@ -11491,36 +11491,36 @@
     </row>
   </sheetData>
   <mergeCells count="30">
+    <mergeCell ref="A4:B4"/>
+    <mergeCell ref="D4:E4"/>
+    <mergeCell ref="G4:H4"/>
+    <mergeCell ref="J4:K4"/>
+    <mergeCell ref="M4:N4"/>
+    <mergeCell ref="P4:Q4"/>
+    <mergeCell ref="S4:T4"/>
+    <mergeCell ref="V4:W4"/>
+    <mergeCell ref="Y4:Z4"/>
+    <mergeCell ref="AB4:AC4"/>
+    <mergeCell ref="AE4:AF4"/>
+    <mergeCell ref="AH4:AI4"/>
+    <mergeCell ref="AK4:AL4"/>
+    <mergeCell ref="AN4:AO4"/>
+    <mergeCell ref="AQ4:AR4"/>
+    <mergeCell ref="A6:B6"/>
+    <mergeCell ref="D6:E6"/>
+    <mergeCell ref="G6:H6"/>
+    <mergeCell ref="J6:K6"/>
+    <mergeCell ref="M6:N6"/>
+    <mergeCell ref="P6:Q6"/>
+    <mergeCell ref="S6:T6"/>
+    <mergeCell ref="V6:W6"/>
+    <mergeCell ref="Y6:Z6"/>
+    <mergeCell ref="AB6:AC6"/>
     <mergeCell ref="AE6:AF6"/>
     <mergeCell ref="AH6:AI6"/>
     <mergeCell ref="AK6:AL6"/>
     <mergeCell ref="AN6:AO6"/>
     <mergeCell ref="AQ6:AR6"/>
-    <mergeCell ref="P6:Q6"/>
-    <mergeCell ref="S6:T6"/>
-    <mergeCell ref="V6:W6"/>
-    <mergeCell ref="Y6:Z6"/>
-    <mergeCell ref="AB6:AC6"/>
-    <mergeCell ref="A6:B6"/>
-    <mergeCell ref="D6:E6"/>
-    <mergeCell ref="G6:H6"/>
-    <mergeCell ref="J6:K6"/>
-    <mergeCell ref="M6:N6"/>
-    <mergeCell ref="AE4:AF4"/>
-    <mergeCell ref="AH4:AI4"/>
-    <mergeCell ref="AK4:AL4"/>
-    <mergeCell ref="AN4:AO4"/>
-    <mergeCell ref="AQ4:AR4"/>
-    <mergeCell ref="P4:Q4"/>
-    <mergeCell ref="S4:T4"/>
-    <mergeCell ref="V4:W4"/>
-    <mergeCell ref="Y4:Z4"/>
-    <mergeCell ref="AB4:AC4"/>
-    <mergeCell ref="A4:B4"/>
-    <mergeCell ref="D4:E4"/>
-    <mergeCell ref="G4:H4"/>
-    <mergeCell ref="J4:K4"/>
-    <mergeCell ref="M4:N4"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>